<commit_message>
Added Phillip Island and Bass Coast. Checked all nest issues and fuzzy matching. Up to joining threat and nest data together
</commit_message>
<xml_diff>
--- a/data/nest_issues_commented/BC_nest_data_issues_220825.xlsx
+++ b/data/nest_issues_commented/BC_nest_data_issues_220825.xlsx
@@ -153,7 +153,7 @@
     <t xml:space="preserve">13122010</t>
   </si>
   <si>
-    <t xml:space="preserve">08012011</t>
+    <t xml:space="preserve">01012011</t>
   </si>
   <si>
     <t xml:space="preserve">signnest,ropefence</t>
@@ -168,7 +168,7 @@
     <t xml:space="preserve">1/2 adult size, fluffy</t>
   </si>
   <si>
-    <t xml:space="preserve">26</t>
+    <t xml:space="preserve">19</t>
   </si>
   <si>
     <t xml:space="preserve">Williamsons Beach Further West</t>
@@ -752,22 +752,22 @@
         <v>50</v>
       </c>
       <c r="P3" s="1" t="n">
-        <v>40551</v>
+        <v>40544</v>
       </c>
       <c r="Q3" s="1" t="n">
         <v>40525</v>
       </c>
       <c r="R3" s="1" t="n">
-        <v>40551</v>
+        <v>40544</v>
       </c>
       <c r="S3" t="n">
         <v>162</v>
       </c>
       <c r="T3" t="n">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="U3" t="n">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>

</xml_diff>